<commit_message>
added fix for missing red and orange tints
</commit_message>
<xml_diff>
--- a/results/summit_financials.xlsx
+++ b/results/summit_financials.xlsx
@@ -753,7 +753,7 @@
       <color/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -780,6 +780,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF6600"/>
       </patternFill>
     </fill>
     <fill>
@@ -837,7 +842,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment wrapText="true"/>
@@ -904,13 +909,16 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="right" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" wrapText="true"/>
     </xf>
   </cellXfs>
@@ -3891,7 +3899,7 @@
         <f>276</f>
         <v>276</v>
       </c>
-      <c r="G18" s="7"/>
+      <c r="G18" s="24"/>
       <c r="H18" s="8">
         <f t="shared" si="3"/>
         <v>554</v>
@@ -3912,7 +3920,7 @@
         <v>563</v>
       </c>
       <c r="F19" s="7"/>
-      <c r="G19" s="24"/>
+      <c r="G19" s="25"/>
       <c r="H19" s="8">
         <f t="shared" si="3"/>
         <v>1042.33</v>
@@ -3933,7 +3941,7 @@
         <f>-552.76</f>
         <v>-552.76</v>
       </c>
-      <c r="G20" s="24"/>
+      <c r="G20" s="25"/>
       <c r="H20" s="8">
         <f t="shared" si="3"/>
         <v>27.9300000000001</v>
@@ -4030,7 +4038,7 @@
         <f t="shared" si="6"/>
         <v>68985.79</v>
       </c>
-      <c r="G23" s="25">
+      <c r="G23" s="26">
         <f t="shared" si="6"/>
         <v>85247.85</v>
       </c>
@@ -4433,7 +4441,7 @@
         <f>856.64</f>
         <v>856.64</v>
       </c>
-      <c r="G37" s="23">
+      <c r="G37" s="22">
         <f>1282.55</f>
         <v>1282.55</v>
       </c>
@@ -4701,7 +4709,7 @@
         <v>469.24</v>
       </c>
       <c r="F47" s="7"/>
-      <c r="G47" s="7"/>
+      <c r="G47" s="24"/>
       <c r="H47" s="8">
         <f t="shared" si="7"/>
         <v>643.85</v>
@@ -4728,7 +4736,7 @@
         <v>78.2</v>
       </c>
       <c r="F48" s="7"/>
-      <c r="G48" s="7"/>
+      <c r="G48" s="24"/>
       <c r="H48" s="8">
         <f t="shared" si="7"/>
         <v>495.65</v>
@@ -4881,7 +4889,7 @@
         <v>27.6</v>
       </c>
       <c r="F54" s="7"/>
-      <c r="G54" s="24"/>
+      <c r="G54" s="25"/>
       <c r="H54" s="8">
         <f t="shared" si="7"/>
         <v>4753.95</v>
@@ -4899,7 +4907,7 @@
       <c r="D55" s="7"/>
       <c r="E55" s="7"/>
       <c r="F55" s="7"/>
-      <c r="G55" s="24"/>
+      <c r="G55" s="25"/>
       <c r="H55" s="8">
         <f t="shared" si="7"/>
         <v>289.22</v>
@@ -4926,7 +4934,7 @@
         <f>90</f>
         <v>90</v>
       </c>
-      <c r="G56" s="26"/>
+      <c r="G56" s="27"/>
       <c r="H56" s="8">
         <f t="shared" si="7"/>
         <v>496.37</v>
@@ -4956,7 +4964,7 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="G57" s="26">
+      <c r="G57" s="27">
         <f>0</f>
         <v>0</v>
       </c>
@@ -5778,7 +5786,7 @@
         <f>4169.16</f>
         <v>4169.16</v>
       </c>
-      <c r="G85" s="24"/>
+      <c r="G85" s="25"/>
       <c r="H85" s="8">
         <f t="shared" si="7"/>
         <v>5069.16</v>
@@ -5889,7 +5897,7 @@
       </c>
       <c r="E89" s="7"/>
       <c r="F89" s="7"/>
-      <c r="G89" s="24"/>
+      <c r="G89" s="25"/>
       <c r="H89" s="8">
         <f t="shared" ref="H89:H98" si="20">(((((B89)+(C89))+(D89))+(E89))+(F89))+(G89)</f>
         <v>1382.5</v>
@@ -5967,7 +5975,7 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="G92" s="26">
+      <c r="G92" s="27">
         <f>0</f>
         <v>0</v>
       </c>
@@ -6224,7 +6232,7 @@
         <f>103.98</f>
         <v>103.98</v>
       </c>
-      <c r="G101" s="24"/>
+      <c r="G101" s="25"/>
       <c r="H101" s="8">
         <f>(((((B101)+(C101))+(D101))+(E101))+(F101))+(G101)</f>
         <v>384.43</v>
@@ -6437,7 +6445,7 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="G109" s="26">
+      <c r="G109" s="27">
         <f>0</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
added number formatting fix for tinted last month cells
</commit_message>
<xml_diff>
--- a/results/summit_financials.xlsx
+++ b/results/summit_financials.xlsx
@@ -903,22 +903,22 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="right" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="4" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" wrapText="true"/>
     </xf>
   </cellXfs>
@@ -4441,7 +4441,7 @@
         <f>856.64</f>
         <v>856.64</v>
       </c>
-      <c r="G37" s="22">
+      <c r="G37" s="23">
         <f>1282.55</f>
         <v>1282.55</v>
       </c>
@@ -5078,7 +5078,7 @@
         <f>100</f>
         <v>100</v>
       </c>
-      <c r="G61" s="22">
+      <c r="G61" s="23">
         <f>100</f>
         <v>100</v>
       </c>

</xml_diff>